<commit_message>
updated documentation for spatially varying demographic rates
</commit_message>
<xml_diff>
--- a/doc/Manual/Batchmode/StageStructFile.xlsx
+++ b/doc/Manual/Batchmode/StageStructFile.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jreeg.IBB\RangeShiftR\transloc_new_genetics_spatial_demog\RangeShifter_batch\doc\Manual\Batchmode\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jreeg.IBB\RangeShiftR\develop\RangeShifter_batch\doc\Manual\Batchmode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEB29F4C-6E2D-49E3-8E0D-8F048EE66B3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEF28E96-17F3-47C7-AA53-95EA2B607AD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19920" yWindow="1800" windowWidth="16875" windowHeight="12900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Description" sheetId="2" r:id="rId1"/>
@@ -22,7 +22,20 @@
     <sheet name="Stage Weights asexual,implicit" sheetId="8" r:id="rId7"/>
     <sheet name="Layer matrix" sheetId="10" r:id="rId8"/>
   </sheets>
-  <calcPr calcId="125725"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -73,7 +86,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="85">
   <si>
     <t>PRep</t>
   </si>
@@ -474,24 +487,15 @@
     <t>Name of the fecundity layer matrix file (*.txt)</t>
   </si>
   <si>
-    <t>Required if fecundity should be spatially varying. Then you need to assign the layer number to the stages, sexes for which fecundity should be spatially varying. Structure: first column stage, second column layer nb for female, third column layer nb for male</t>
-  </si>
-  <si>
     <t>Name of the fdevelopment layer matrix file (*.txt)</t>
   </si>
   <si>
-    <t>Required if development should be spatially varying. Then you need to assign the layer number to the stages, sexes for which fecundity should be spatially varying. Structure: first column stage, second column layer nb for female, third column layer nb for male</t>
-  </si>
-  <si>
     <t>SurvLayerFile</t>
   </si>
   <si>
     <t>Name of the survival layer matrix file (*.txt)</t>
   </si>
   <si>
-    <t>Required if survival should be spatially varying. Then you need to assign the layer number to the stages, sexes for which fecundity should be spatially varying. Structure: first column stage, second column layer nb for female, third column layer nb for male</t>
-  </si>
-  <si>
     <t>Stage</t>
   </si>
   <si>
@@ -501,9 +505,6 @@
     <t>male layer</t>
   </si>
   <si>
-    <t>FeyLayerFile</t>
-  </si>
-  <si>
     <t>feclayer.txt</t>
   </si>
   <si>
@@ -511,6 +512,15 @@
   </si>
   <si>
     <t>survlayer.txt</t>
+  </si>
+  <si>
+    <t>Required if fecundity should be spatially varying. Then you need to assign the layer number to the stages, sexes for which fecundity should be spatially varying. Structure: first column stage, second column layer nb for female, third column layer nb for male. If fecundity for a stage/sex is not spatially varying, a value of -9 will set the fecundity to the maximal rate provided in the transition matrix file.</t>
+  </si>
+  <si>
+    <t>Required if development should be spatially varying. Then you need to assign the layer number to the stages, sexes for which fecundity should be spatially varying. Structure: first column stage, second column layer nb for female, third column layer nb for male. If development rate for a stage/sex is not spatially varying, a value of -9 will set  the development rate to the maximal rate provided in the transition matrix file.</t>
+  </si>
+  <si>
+    <t>Required if survival should be spatially varying. Then you need to assign the layer number to the stages, sexes for which fecundity should be spatially varying. Structure: first column stage, second column layer nb for female, third column layer nb for male. If survival rate for a stage/sex is not spatially varying, a value of -9 will set the survival rate to the maximal rate provided in the transition matrix file.</t>
   </si>
 </sst>
 </file>
@@ -1022,16 +1032,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D22"/>
-  <sheetFormatPr defaultColWidth="9.08984375" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.6328125" style="7" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.6328125" style="7" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="65.90625" style="7" customWidth="1"/>
-    <col min="4" max="4" width="46.6328125" style="7" bestFit="1" customWidth="1"/>
-    <col min="5" max="16384" width="9.08984375" style="7"/>
+    <col min="1" max="1" width="16.5703125" style="7" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.5703125" style="7" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="65.85546875" style="7" customWidth="1"/>
+    <col min="4" max="4" width="46.5703125" style="7" bestFit="1" customWidth="1"/>
+    <col min="5" max="16384" width="9.140625" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>46</v>
       </c>
@@ -1045,7 +1055,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
         <v>12</v>
       </c>
@@ -1059,7 +1069,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
         <v>59</v>
       </c>
@@ -1073,7 +1083,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>0</v>
       </c>
@@ -1085,7 +1095,7 @@
       </c>
       <c r="D4" s="9"/>
     </row>
-    <row r="5" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
         <v>2</v>
       </c>
@@ -1097,7 +1107,7 @@
       </c>
       <c r="D5" s="9"/>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
         <v>3</v>
       </c>
@@ -1109,7 +1119,7 @@
       </c>
       <c r="D6" s="9"/>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
         <v>41</v>
       </c>
@@ -1121,7 +1131,7 @@
       </c>
       <c r="D7" s="9"/>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
         <v>25</v>
       </c>
@@ -1133,7 +1143,7 @@
       </c>
       <c r="D8" s="9"/>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
         <v>13</v>
       </c>
@@ -1145,7 +1155,7 @@
       </c>
       <c r="D9" s="9"/>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
         <v>14</v>
       </c>
@@ -1157,7 +1167,7 @@
       </c>
       <c r="D10" s="10"/>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
         <v>15</v>
       </c>
@@ -1171,7 +1181,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" ht="135" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
         <v>70</v>
       </c>
@@ -1182,10 +1192,10 @@
         <v>72</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
         <v>16</v>
       </c>
@@ -1197,7 +1207,7 @@
       </c>
       <c r="D13" s="9"/>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
         <v>17</v>
       </c>
@@ -1211,7 +1221,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
         <v>18</v>
       </c>
@@ -1223,7 +1233,7 @@
       </c>
       <c r="D15" s="10"/>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
         <v>19</v>
       </c>
@@ -1237,7 +1247,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" ht="135" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
         <v>71</v>
       </c>
@@ -1245,13 +1255,13 @@
         <v>44</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
         <v>20</v>
       </c>
@@ -1263,7 +1273,7 @@
       </c>
       <c r="D18" s="9"/>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
         <v>21</v>
       </c>
@@ -1277,7 +1287,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
         <v>22</v>
       </c>
@@ -1289,7 +1299,7 @@
       </c>
       <c r="D20" s="10"/>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
         <v>23</v>
       </c>
@@ -1303,18 +1313,18 @@
         <v>69</v>
       </c>
     </row>
-    <row r="22" spans="1:4" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:4" ht="135" x14ac:dyDescent="0.25">
       <c r="A22" s="7" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B22" s="9" t="s">
         <v>44</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="D22" s="10" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -1326,31 +1336,31 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:U14"/>
-  <sheetFormatPr defaultColWidth="9.08984375" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.54296875" style="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.36328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.08984375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.6328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.08984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.36328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.6328125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.6328125" customWidth="1"/>
-    <col min="12" max="12" width="12.453125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.90625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12.6328125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="16.08984375" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="16.08984375" customWidth="1"/>
-    <col min="17" max="17" width="12.90625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="14.36328125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="13.36328125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="16.54296875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.5703125" customWidth="1"/>
+    <col min="12" max="12" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="16.140625" customWidth="1"/>
+    <col min="17" max="17" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="16.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:21" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
         <v>12</v>
       </c>
@@ -1382,7 +1392,7 @@
         <v>15</v>
       </c>
       <c r="K1" s="13" t="s">
-        <v>82</v>
+        <v>70</v>
       </c>
       <c r="L1" s="13" t="s">
         <v>16</v>
@@ -1412,10 +1422,10 @@
         <v>23</v>
       </c>
       <c r="U1" s="11" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.35">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1480,7 +1490,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1545,7 +1555,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1610,7 +1620,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1675,7 +1685,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1740,7 +1750,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1805,7 +1815,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1870,7 +1880,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1935,7 +1945,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -2000,7 +2010,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -2065,7 +2075,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -2130,7 +2140,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -2195,18 +2205,18 @@
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="O14" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="T14" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
     </row>
   </sheetData>
@@ -2218,9 +2228,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FD70802-07FD-4D0F-9BFE-8A3084CA253C}">
   <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>38</v>
       </c>
@@ -2234,7 +2244,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>0</v>
       </c>
@@ -2248,7 +2258,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
@@ -2270,26 +2280,26 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.36328125" customWidth="1"/>
+    <col min="1" max="1" width="10.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B1" s="15"/>
       <c r="C1" s="15"/>
       <c r="D1" s="15"/>
       <c r="E1" s="15"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="16"/>
       <c r="E2" s="2"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="16"/>
       <c r="E3" s="2"/>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="16"/>
     </row>
   </sheetData>
@@ -2300,12 +2310,12 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:H6"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.36328125" customWidth="1"/>
+    <col min="1" max="1" width="10.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
         <v>38</v>
       </c>
@@ -2331,7 +2341,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
         <v>40</v>
       </c>
@@ -2357,7 +2367,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
         <v>8</v>
       </c>
@@ -2383,7 +2393,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
         <v>9</v>
       </c>
@@ -2409,7 +2419,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
         <v>10</v>
       </c>
@@ -2435,7 +2445,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
         <v>11</v>
       </c>
@@ -2469,9 +2479,9 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:G7"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
         <v>39</v>
       </c>
@@ -2494,7 +2504,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
         <v>35</v>
       </c>
@@ -2517,7 +2527,7 @@
         <v>2.5</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
         <v>36</v>
       </c>
@@ -2540,7 +2550,7 @@
         <v>2.5</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
         <v>8</v>
       </c>
@@ -2563,7 +2573,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
         <v>9</v>
       </c>
@@ -2586,7 +2596,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
         <v>10</v>
       </c>
@@ -2609,7 +2619,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
         <v>11</v>
       </c>
@@ -2641,9 +2651,9 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:D4"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
         <v>39</v>
       </c>
@@ -2657,7 +2667,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="16">
         <v>0</v>
       </c>
@@ -2671,7 +2681,7 @@
         <v>2.5</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="16">
         <v>1</v>
       </c>
@@ -2685,7 +2695,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="16">
         <v>2</v>
       </c>
@@ -2708,20 +2718,24 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{252DAFEA-46EE-4355-AB33-D06CE53A4392}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.28515625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="B1" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="C1" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>0</v>
       </c>
@@ -2732,7 +2746,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
@@ -2743,7 +2757,7 @@
         <v>-9</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2</v>
       </c>

</xml_diff>